<commit_message>
Market changes for USA
</commit_message>
<xml_diff>
--- a/frontend/public/template/Portfolio_AI_Template_IND.xlsx
+++ b/frontend/public/template/Portfolio_AI_Template_IND.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\AI\git\portfolio_ai\frontend\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1882A3EF-4AE7-48CB-AE9A-9A0EE3251C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1A738B-71F9-4D36-A14F-DF86E29069B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Investor" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Name</t>
   </si>
@@ -54,9 +54,6 @@
     <t>SBIN</t>
   </si>
   <si>
-    <t>BSE</t>
-  </si>
-  <si>
     <t>Fund Name</t>
   </si>
   <si>
@@ -91,6 +88,18 @@
   </si>
   <si>
     <t>satheeshkumartest@gmail.com</t>
+  </si>
+  <si>
+    <t>HDFCBANK</t>
+  </si>
+  <si>
+    <t>ADANIPOWER</t>
+  </si>
+  <si>
+    <t>ICICIBANK</t>
+  </si>
+  <si>
+    <t>RVNL</t>
   </si>
 </sst>
 </file>
@@ -106,23 +115,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -130,17 +145,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -446,97 +477,157 @@
   <cols>
     <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{E2A3AEB0-281C-426D-81BF-581927352146}"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.33203125" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.5546875" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>10</v>
       </c>
-      <c r="D2">
-        <v>3500</v>
+      <c r="D2" s="1">
+        <v>2200</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>5</v>
       </c>
-      <c r="D3">
-        <v>2800</v>
+      <c r="D3" s="1">
+        <v>1400</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1">
+        <v>20</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="4">
         <v>10</v>
       </c>
-      <c r="C4">
-        <v>20</v>
-      </c>
-      <c r="D4">
-        <v>800</v>
+      <c r="D5" s="4">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="4">
+        <v>70</v>
+      </c>
+      <c r="D6" s="4">
+        <v>153.09</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="4">
+        <v>10</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1321.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="4">
+        <v>150</v>
+      </c>
+      <c r="D8" s="4">
+        <v>200.1</v>
       </c>
     </row>
   </sheetData>
@@ -549,51 +640,51 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="44.44140625" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="1">
+        <v>100</v>
+      </c>
+      <c r="D2" s="1">
+        <v>34.880000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2">
-        <v>100</v>
-      </c>
-      <c r="D2">
-        <v>34.880000000000003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>50</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>90</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Market changes for USA sector updated
</commit_message>
<xml_diff>
--- a/frontend/public/template/Portfolio_AI_Template_IND.xlsx
+++ b/frontend/public/template/Portfolio_AI_Template_IND.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\AI\git\portfolio_ai\frontend\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1A738B-71F9-4D36-A14F-DF86E29069B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1948CAD4-92A4-4123-BDEC-91EE3BE97209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
   <si>
     <t>Name</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>RVNL</t>
+  </si>
+  <si>
+    <t>BSE</t>
   </si>
 </sst>
 </file>
@@ -164,12 +167,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,7 +539,7 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1">
         <v>10</v>
@@ -575,58 +577,58 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="1">
         <v>10</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="1">
         <v>815</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="1">
         <v>70</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="1">
         <v>153.09</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="1">
         <v>10</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="1">
         <v>1321.4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="1">
         <v>150</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="1">
         <v>200.1</v>
       </c>
     </row>

</xml_diff>